<commit_message>
#7 Client and JLCPCB BOM updated.
</commit_message>
<xml_diff>
--- a/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/Client_BOM_PowerCutMonitor-v1.1.xlsx
+++ b/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/Client_BOM_PowerCutMonitor-v1.1.xlsx
@@ -129,9 +129,6 @@
     <t>Q3</t>
   </si>
   <si>
-    <t>R1, R2, R3</t>
-  </si>
-  <si>
     <t>R4, R5, R7</t>
   </si>
   <si>
@@ -150,9 +147,6 @@
     <t>SW1</t>
   </si>
   <si>
-    <t>SW2, SW3</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -514,6 +508,12 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>SW2, SW3, SW4</t>
+  </si>
+  <si>
+    <t>R1, R2, R3, R15</t>
   </si>
 </sst>
 </file>
@@ -1046,25 +1046,25 @@
         <v>17</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1080,19 +1080,19 @@
         <v>18</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1112,19 +1112,19 @@
         <v>19</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J4" s="9">
         <v>4</v>
@@ -1144,19 +1144,19 @@
         <v>20</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1176,19 +1176,19 @@
         <v>21</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1208,19 +1208,19 @@
         <v>22</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
@@ -1240,19 +1240,19 @@
         <v>23</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1272,19 +1272,19 @@
         <v>24</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
@@ -1304,19 +1304,19 @@
         <v>25</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
@@ -1336,19 +1336,19 @@
         <v>26</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1368,19 +1368,19 @@
         <v>27</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>
@@ -1400,19 +1400,19 @@
         <v>28</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1432,19 +1432,19 @@
         <v>29</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1464,19 +1464,19 @@
         <v>30</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1496,19 +1496,19 @@
         <v>31</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1528,19 +1528,19 @@
         <v>32</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1560,19 +1560,19 @@
         <v>33</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1592,19 +1592,19 @@
         <v>34</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J19" s="7">
         <v>2</v>
@@ -1624,19 +1624,19 @@
         <v>35</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1653,25 +1653,25 @@
         <v>12</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>36</v>
+        <v>164</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J21" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K21" s="7"/>
     </row>
@@ -1685,22 +1685,22 @@
         <v>12</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J22" s="9">
         <v>3</v>
@@ -1717,22 +1717,22 @@
         <v>12</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1749,22 +1749,22 @@
         <v>12</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -1779,22 +1779,22 @@
       </c>
       <c r="C25" s="12"/>
       <c r="D25" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -1811,22 +1811,22 @@
         <v>12</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J26" s="9">
         <v>3</v>
@@ -1843,22 +1843,22 @@
         <v>13</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1875,25 +1875,25 @@
         <v>13</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>43</v>
+        <v>163</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J28" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K28" s="9"/>
     </row>
@@ -1907,22 +1907,22 @@
         <v>14</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -1939,22 +1939,22 @@
         <v>15</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -1971,22 +1971,22 @@
         <v>15</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2003,22 +2003,22 @@
         <v>16</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>

</xml_diff>

<commit_message>
#7 #5 U3 Part number updated in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/Client_BOM_PowerCutMonitor-v1.1.xlsx
+++ b/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/Client_BOM_PowerCutMonitor-v1.1.xlsx
@@ -1,20 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\davetetlow-PowerCutMonitor\Design-Files\PowerCutMonitor-v1.1 (Contactless Version)\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2E2EB4-5191-4C75-9AF2-8D5E7B400226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -270,9 +282,6 @@
     <t>IC REG BUCK 3.3V 2A TSOT26</t>
   </si>
   <si>
-    <t>IC FF D-TYPE SINGLE 4BIT 16PDIP</t>
-  </si>
-  <si>
     <t>32.768kHz Surface Mount Crystal 12.5pF ±20ppm SMD3215-2P Crystals ROHS</t>
   </si>
   <si>
@@ -342,9 +351,6 @@
     <t>TSOT-23-6</t>
   </si>
   <si>
-    <t>PDIP-16</t>
-  </si>
-  <si>
     <t>SMD3215-2P</t>
   </si>
   <si>
@@ -426,9 +432,6 @@
     <t>AP63203WU-7</t>
   </si>
   <si>
-    <t>CD40175BE</t>
-  </si>
-  <si>
     <t>Q13FC13500004</t>
   </si>
   <si>
@@ -486,9 +489,6 @@
     <t>Espressif Systems</t>
   </si>
   <si>
-    <t>Texas Instruments</t>
-  </si>
-  <si>
     <t>Epson</t>
   </si>
   <si>
@@ -553,12 +553,24 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>CD4017BE(LX)</t>
+  </si>
+  <si>
+    <t>lingxingic</t>
+  </si>
+  <si>
+    <t>DIP-16</t>
+  </si>
+  <si>
+    <t>Rising Edge 3V~15V 1 11MHz DIP-16 Counters, Dividers ROHS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1043,7 +1055,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1051,7 +1063,7 @@
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="5" max="5" width="48.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
@@ -1088,22 +1100,22 @@
         <v>51</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1122,16 +1134,16 @@
         <v>52</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1154,16 +1166,16 @@
         <v>53</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="J4" s="9">
         <v>4</v>
@@ -1186,16 +1198,16 @@
         <v>54</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1218,16 +1230,16 @@
         <v>55</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1250,16 +1262,16 @@
         <v>56</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
@@ -1282,16 +1294,16 @@
         <v>57</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1314,16 +1326,16 @@
         <v>58</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
@@ -1346,16 +1358,16 @@
         <v>59</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
@@ -1378,16 +1390,16 @@
         <v>60</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1410,16 +1422,16 @@
         <v>61</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>
@@ -1442,16 +1454,16 @@
         <v>62</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1474,16 +1486,16 @@
         <v>63</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1506,16 +1518,16 @@
         <v>64</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1538,16 +1550,16 @@
         <v>65</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1570,16 +1582,16 @@
         <v>66</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1602,16 +1614,16 @@
         <v>67</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1634,16 +1646,16 @@
         <v>68</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1666,16 +1678,16 @@
         <v>69</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J20" s="9">
         <v>2</v>
@@ -1698,16 +1710,16 @@
         <v>70</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1730,16 +1742,16 @@
         <v>71</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J22" s="9">
         <v>2</v>
@@ -1762,16 +1774,16 @@
         <v>72</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="J23" s="7">
         <v>4</v>
@@ -1794,16 +1806,16 @@
         <v>73</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="J24" s="9">
         <v>3</v>
@@ -1826,16 +1838,16 @@
         <v>74</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -1858,16 +1870,16 @@
         <v>75</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -1888,16 +1900,16 @@
         <v>76</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1920,16 +1932,16 @@
         <v>77</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="J28" s="9">
         <v>3</v>
@@ -1952,16 +1964,16 @@
         <v>78</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="J29" s="7">
         <v>4</v>
@@ -1984,16 +1996,16 @@
         <v>79</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2016,16 +2028,16 @@
         <v>80</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J31" s="7">
         <v>3</v>
@@ -2048,16 +2060,16 @@
         <v>81</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2080,16 +2092,16 @@
         <v>82</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2109,19 +2121,19 @@
         <v>49</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>83</v>
+        <v>177</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>107</v>
+        <v>176</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2141,19 +2153,19 @@
         <v>50</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="I35" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>

</xml_diff>

<commit_message>
#7 BOM Minor resistors, capacitor update. No effect on PCB design
</commit_message>
<xml_diff>
--- a/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/Client_BOM_PowerCutMonitor-v1.1.xlsx
+++ b/Design-Files/PowerCutMonitor-v1.1 (Contactless Version)/BOM/Client_BOM_PowerCutMonitor-v1.1.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\davetetlow-PowerCutMonitor\Design-Files\PowerCutMonitor-v1.1 (Contactless Version)\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A69968A-029D-428F-87A4-5EFA96CB62F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="6900"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -194,15 +198,6 @@
     <t>C15</t>
   </si>
   <si>
-    <t>CAP TANT 33UF 10% 10V 1411</t>
-  </si>
-  <si>
-    <t>TAJB336K010RNJ</t>
-  </si>
-  <si>
-    <t>33uF</t>
-  </si>
-  <si>
     <t>Diode</t>
   </si>
   <si>
@@ -413,9 +408,6 @@
     <t>2.2K</t>
   </si>
   <si>
-    <t>R5, R7</t>
-  </si>
-  <si>
     <t>RES 1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -437,9 +429,6 @@
     <t>47K</t>
   </si>
   <si>
-    <t>R8</t>
-  </si>
-  <si>
     <t>RES 4.7K OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -461,9 +450,6 @@
     <t>18K</t>
   </si>
   <si>
-    <t>R12, R13, R14</t>
-  </si>
-  <si>
     <t>RES 100K OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -497,9 +483,6 @@
     <t>RC0402FR-070RL</t>
   </si>
   <si>
-    <t>0R</t>
-  </si>
-  <si>
     <t>Switch</t>
   </si>
   <si>
@@ -588,19 +571,34 @@
   </si>
   <si>
     <t>Epson</t>
+  </si>
+  <si>
+    <t>47uF</t>
+  </si>
+  <si>
+    <t>TPSB476K010R0250</t>
+  </si>
+  <si>
+    <t>CAP TANT 47UF 10% 10V 1411</t>
+  </si>
+  <si>
+    <t>R5, R7, R10</t>
+  </si>
+  <si>
+    <t>R13, R14</t>
+  </si>
+  <si>
+    <t>R8, R12</t>
+  </si>
+  <si>
+    <t>DNP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -644,151 +642,31 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -807,194 +685,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1085,253 +777,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1371,68 +821,36 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1690,28 +1108,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="9.85714285714286" customWidth="1"/>
-    <col min="7" max="7" width="27.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" customWidth="1"/>
+    <col min="7" max="7" width="27.33203125" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="6.71428571428571" customWidth="1"/>
-    <col min="10" max="10" width="9.28571428571429" customWidth="1"/>
-    <col min="11" max="11" width="9.14285714285714" customWidth="1"/>
+    <col min="9" max="9" width="6.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.33203125" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1724,7 +1143,7 @@
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
     </row>
-    <row r="2" ht="15.75" spans="1:11">
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1757,10 +1176,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="15.75" spans="1:11">
+    <row r="3" spans="1:11">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
-        <f>ROW(B3)-ROW($B$2)</f>
+        <f t="shared" ref="B3:B37" si="0">ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -1789,10 +1208,10 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" ht="15.75" spans="1:11">
+    <row r="4" spans="1:11">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
-        <f>ROW(B4)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -1821,10 +1240,10 @@
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" ht="15.75" spans="1:11">
+    <row r="5" spans="1:11">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
-        <f>ROW(B5)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="8" t="s">
@@ -1853,10 +1272,10 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" ht="15.75" spans="1:11">
+    <row r="6" spans="1:11">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
-        <f>ROW(B6)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -1885,10 +1304,10 @@
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="15.75" spans="1:11">
+    <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
-        <f>ROW(B7)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
@@ -1917,10 +1336,10 @@
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" ht="15.75" spans="1:11">
+    <row r="8" spans="1:11">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
-        <f>ROW(B8)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
@@ -1949,10 +1368,10 @@
       </c>
       <c r="K8" s="12"/>
     </row>
-    <row r="9" ht="15.75" spans="1:11">
+    <row r="9" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
-        <f>ROW(B9)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
@@ -1981,10 +1400,10 @@
       </c>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" ht="15.75" spans="1:11">
+    <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
-        <f>ROW(B10)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -2016,7 +1435,7 @@
     <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
-        <f>ROW(B11)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="8" t="s">
@@ -2026,51 +1445,51 @@
         <v>54</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>55</v>
+        <v>182</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>37</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>56</v>
+        <v>181</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>15</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>57</v>
+        <v>180</v>
       </c>
       <c r="J11" s="9">
         <v>1</v>
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" ht="24.75" spans="1:11">
+    <row r="12" spans="1:11" ht="24">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
-        <f>ROW(B12)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="G12" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="H12" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="I12" s="13" t="s">
         <v>61</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="I12" s="13" t="s">
-        <v>64</v>
       </c>
       <c r="J12" s="12">
         <v>2</v>
@@ -2080,93 +1499,93 @@
     <row r="13" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
-        <f>ROW(B13)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D13" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="H13" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>69</v>
-      </c>
       <c r="I13" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J13" s="9">
         <v>1</v>
       </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" ht="36.75" spans="1:11">
+    <row r="14" spans="1:11" ht="36">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
-        <f>ROW(B14)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="G14" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="H14" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>75</v>
-      </c>
       <c r="I14" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J14" s="12">
         <v>1</v>
       </c>
       <c r="K14" s="12"/>
     </row>
-    <row r="15" ht="24.75" spans="1:11">
+    <row r="15" spans="1:11" ht="24">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
-        <f>ROW(B15)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="H15" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E15" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>80</v>
-      </c>
       <c r="I15" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J15" s="9">
         <v>1</v>
@@ -2176,221 +1595,221 @@
     <row r="16" spans="1:11">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
-        <f>ROW(B16)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G16" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="H16" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="I16" s="13" t="s">
         <v>83</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="I16" s="13" t="s">
-        <v>86</v>
       </c>
       <c r="J16" s="12">
         <v>1</v>
       </c>
       <c r="K16" s="12"/>
     </row>
-    <row r="17" ht="24.75" spans="1:11">
+    <row r="17" spans="1:11" ht="24">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
-        <f>ROW(B17)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="G17" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="H17" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F17" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>92</v>
-      </c>
       <c r="I17" s="10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J17" s="9">
         <v>1</v>
       </c>
       <c r="K17" s="9"/>
     </row>
-    <row r="18" ht="48.75" spans="1:11">
+    <row r="18" spans="1:11" ht="48">
       <c r="A18" s="2"/>
       <c r="B18" s="7">
-        <f>ROW(B18)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D18" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H18" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>96</v>
-      </c>
       <c r="I18" s="10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J18" s="12">
         <v>1</v>
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" ht="36.75" spans="1:11">
+    <row r="19" spans="1:11" ht="36">
       <c r="A19" s="2"/>
       <c r="B19" s="7">
-        <f>ROW(B19)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F19" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="G19" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="H19" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="F19" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>102</v>
-      </c>
       <c r="I19" s="10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J19" s="9">
         <v>1</v>
       </c>
       <c r="K19" s="9"/>
     </row>
-    <row r="20" ht="24.75" spans="1:11">
+    <row r="20" spans="1:11" ht="24">
       <c r="A20" s="2"/>
       <c r="B20" s="7">
-        <f>ROW(B20)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F20" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="G20" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="E20" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="G20" s="13" t="s">
-        <v>107</v>
-      </c>
       <c r="H20" s="12" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J20" s="12">
         <v>2</v>
       </c>
       <c r="K20" s="12"/>
     </row>
-    <row r="21" ht="48.75" spans="1:11">
+    <row r="21" spans="1:11" ht="48">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
-        <f>ROW(B21)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D21" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G21" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="H21" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>112</v>
-      </c>
       <c r="I21" s="10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J21" s="9">
         <v>1</v>
       </c>
       <c r="K21" s="9"/>
     </row>
-    <row r="22" ht="36.75" spans="1:11">
+    <row r="22" spans="1:11" ht="36">
       <c r="A22" s="2"/>
       <c r="B22" s="7">
-        <f>ROW(B22)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D22" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="G22" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="H22" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F22" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="G22" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>117</v>
-      </c>
       <c r="I22" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J22" s="12">
         <v>2</v>
@@ -2400,29 +1819,29 @@
     <row r="23" spans="1:11">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
-        <f>ROW(B23)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="G23" s="10" t="s">
         <v>119</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>122</v>
       </c>
       <c r="H23" s="9" t="s">
         <v>28</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="J23" s="9">
         <v>6</v>
@@ -2432,29 +1851,29 @@
     <row r="24" spans="1:11">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
-        <f>ROW(B24)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="F24" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="D24" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>121</v>
-      </c>
       <c r="G24" s="13" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="H24" s="12" t="s">
         <v>28</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="J24" s="12">
         <v>3</v>
@@ -2464,61 +1883,61 @@
     <row r="25" spans="1:11">
       <c r="A25" s="2"/>
       <c r="B25" s="7">
-        <f>ROW(B25)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F25" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D25" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>121</v>
-      </c>
       <c r="G25" s="10" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>28</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="J25" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" s="9"/>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
-        <f>ROW(B26)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="F26" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="D26" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>121</v>
-      </c>
       <c r="G26" s="13" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H26" s="12" t="s">
         <v>28</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J26" s="12">
         <v>1</v>
@@ -2528,61 +1947,61 @@
     <row r="27" spans="1:11">
       <c r="A27" s="2"/>
       <c r="B27" s="7">
-        <f>ROW(B27)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="F27" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D27" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>121</v>
-      </c>
       <c r="G27" s="10" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="H27" s="9" t="s">
         <v>28</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="J27" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K27" s="9"/>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
-        <f>ROW(B28)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="F28" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="F28" s="12" t="s">
-        <v>121</v>
-      </c>
       <c r="G28" s="13" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="H28" s="12" t="s">
         <v>28</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="J28" s="12">
         <v>1</v>
@@ -2592,157 +2011,157 @@
     <row r="29" spans="1:11">
       <c r="A29" s="2"/>
       <c r="B29" s="7">
-        <f>ROW(B29)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="F29" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>121</v>
-      </c>
       <c r="G29" s="10" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="H29" s="9" t="s">
         <v>28</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="J29" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" s="9"/>
     </row>
-    <row r="30" ht="15.75" spans="1:11">
+    <row r="30" spans="1:11">
       <c r="A30" s="2"/>
       <c r="B30" s="7">
-        <f>ROW(B30)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="F30" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>121</v>
-      </c>
       <c r="G30" s="13" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="H30" s="12" t="s">
         <v>28</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="J30" s="12">
         <v>2</v>
       </c>
       <c r="K30" s="12"/>
     </row>
-    <row r="31" ht="15.75" spans="1:11">
+    <row r="31" spans="1:11">
       <c r="A31" s="2"/>
       <c r="B31" s="7">
-        <f>ROW(B31)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C31" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="G31" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="H31" s="9" t="s">
+      <c r="C31" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="H31" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="I31" s="10" t="s">
-        <v>156</v>
+      <c r="I31" s="15" t="s">
+        <v>186</v>
       </c>
       <c r="J31" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K31" s="9"/>
     </row>
-    <row r="32" ht="36.75" spans="1:11">
+    <row r="32" spans="1:11" ht="36">
       <c r="A32" s="2"/>
       <c r="B32" s="7">
-        <f>ROW(B32)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="I32" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J32" s="12">
         <v>1</v>
       </c>
       <c r="K32" s="12"/>
     </row>
-    <row r="33" ht="15.75" spans="1:11">
+    <row r="33" spans="1:11">
       <c r="A33" s="2"/>
       <c r="B33" s="7">
-        <f>ROW(B33)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G33" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="F33" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>164</v>
-      </c>
       <c r="H33" s="9" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="I33" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J33" s="9">
         <v>3</v>
@@ -2752,29 +2171,29 @@
     <row r="34" spans="1:11">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
-        <f>ROW(B34)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I34" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J34" s="12">
         <v>1</v>
@@ -2784,93 +2203,93 @@
     <row r="35" spans="1:11">
       <c r="A35" s="2"/>
       <c r="B35" s="7">
-        <f>ROW(B35)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I35" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J35" s="9">
         <v>1</v>
       </c>
       <c r="K35" s="9"/>
     </row>
-    <row r="36" ht="24.75" spans="1:11">
+    <row r="36" spans="1:11" ht="24">
       <c r="A36" s="2"/>
       <c r="B36" s="7">
-        <f>ROW(B36)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C36" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="F36" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="D36" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="F36" s="12" t="s">
-        <v>178</v>
-      </c>
       <c r="G36" s="13" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="I36" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J36" s="12">
         <v>1</v>
       </c>
       <c r="K36" s="12"/>
     </row>
-    <row r="37" ht="36.75" spans="1:11">
+    <row r="37" spans="1:11" ht="24">
       <c r="A37" s="2"/>
       <c r="B37" s="7">
-        <f>ROW(B37)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="I37" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J37" s="9">
         <v>1</v>
@@ -2882,7 +2301,6 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>